<commit_message>
updating figure formatting following review
</commit_message>
<xml_diff>
--- a/data/planetary_boundaries_data.xlsx
+++ b/data/planetary_boundaries_data.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\uol.le.ac.uk\root\staff\home\t\twwh1\My Documents\GitHub\planetary_boundaries_plots\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twwh1\GitHub\planetary_boundaries_plots\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D269EE31-45F4-47E7-8BBC-920600A217F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D232CAD-C606-47A1-BB82-5AD34CEFF7C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="1" xr2:uid="{9645B8C2-294A-4B6F-9D52-808A1D49E06C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="2" xr2:uid="{9645B8C2-294A-4B6F-9D52-808A1D49E06C}"/>
   </bookViews>
   <sheets>
     <sheet name="2023" sheetId="1" r:id="rId1"/>
     <sheet name="2025" sheetId="2" r:id="rId2"/>
+    <sheet name="PTME" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,15 +31,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="61">
   <si>
     <t>Climate change</t>
   </si>
@@ -434,6 +432,18 @@
   </si>
   <si>
     <t>following PBS 2025 using the regional boundary values</t>
+  </si>
+  <si>
+    <t>following Barnosky et al 2011 this would be between 0.2 to 9 E/MSY; here we convert a 95% species extinction (Foster et al 2018) to E/MSY assuming a 60 kyr duration for the extinction</t>
+  </si>
+  <si>
+    <t>Functional integrity: measured as energy available to ecosystems (NPP) using loss of terrestrial productivity</t>
+  </si>
+  <si>
+    <t>% reduction in terrestrial NPP</t>
+  </si>
+  <si>
+    <t>following Xu et al 2025</t>
   </si>
 </sst>
 </file>
@@ -443,7 +453,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -477,6 +487,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -495,48 +513,56 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -553,9 +579,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -593,7 +619,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -699,7 +725,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -841,7 +867,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1399,7 +1425,7 @@
       <c r="G6" s="11">
         <v>263</v>
       </c>
-      <c r="H6" s="13">
+      <c r="H6" s="12">
         <v>285.7</v>
       </c>
     </row>
@@ -1425,7 +1451,7 @@
       <c r="G7" s="11">
         <v>2.5</v>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="12">
         <v>2.84</v>
       </c>
     </row>
@@ -1480,7 +1506,7 @@
       <c r="G9" s="11">
         <v>82</v>
       </c>
-      <c r="H9" s="13">
+      <c r="H9" s="12">
         <v>165</v>
       </c>
     </row>
@@ -1558,7 +1584,7 @@
       <c r="G12" s="11">
         <v>50</v>
       </c>
-      <c r="H12" s="13">
+      <c r="H12" s="12">
         <v>22</v>
       </c>
     </row>
@@ -1621,4 +1647,305 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1F638F2-7F4F-4BFD-A707-7DDFC891A314}">
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="29.90625" style="15" customWidth="1"/>
+    <col min="2" max="8" width="19.81640625" style="15" customWidth="1"/>
+    <col min="9" max="9" width="33" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="13"/>
+    </row>
+    <row r="3" spans="1:9" ht="58" x14ac:dyDescent="0.35">
+      <c r="A3" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="13"/>
+    </row>
+    <row r="4" spans="1:9" ht="87" x14ac:dyDescent="0.35">
+      <c r="A4" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="11">
+        <v>1</v>
+      </c>
+      <c r="F4" s="11">
+        <v>10</v>
+      </c>
+      <c r="G4" s="11">
+        <v>100</v>
+      </c>
+      <c r="H4" s="11">
+        <v>15.83</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="87" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="11">
+        <v>1.9</v>
+      </c>
+      <c r="F5" s="11">
+        <v>10</v>
+      </c>
+      <c r="G5" s="11">
+        <v>20</v>
+      </c>
+      <c r="H5" s="11">
+        <v>70</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="13"/>
+    </row>
+    <row r="7" spans="1:9" ht="87" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="13"/>
+    </row>
+    <row r="8" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+    </row>
+    <row r="9" spans="1:9" ht="58" x14ac:dyDescent="0.35">
+      <c r="A9" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="13"/>
+    </row>
+    <row r="10" spans="1:9" ht="116" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="11"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="13"/>
+    </row>
+    <row r="12" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="13"/>
+    </row>
+    <row r="13" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+    </row>
+    <row r="14" spans="1:9" ht="87" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>